<commit_message>
fix(billing): update bank account to GPPM TING TING company account
Update static bank details (Chủ Tài Khoản / Số Tài Khoản) across all
template sources:
- email_template.go (sao-kê email, HTML + text body)
- payroll_statement.html (payroll statement email)
- sao_ke_tt_theo_du_an.xlsx, payroll_template.xlsx (Excel exports)

Old: NGUYEN VIET DUNG / 1357210887
New: CONG TY TNHH MTV GPPM TING TING / 283866888
Bank unchanged: TECHCOMBANK
</commit_message>
<xml_diff>
--- a/backend/templates/payroll_template.xlsx
+++ b/backend/templates/payroll_template.xlsx
@@ -63,13 +63,13 @@
     <t>Chủ Tài Khoản</t>
   </si>
   <si>
-    <t>NGUYEN VIET DUNG</t>
+    <t>CONG TY TNHH MTV GPPM TING TING</t>
   </si>
   <si>
     <t>Số Tài Khoản</t>
   </si>
   <si>
-    <t>1357210887</t>
+    <t>283866888</t>
   </si>
   <si>
     <t>Ngân Hàng</t>

</xml_diff>

<commit_message>
fix(payroll): adjust Excel templates to preserve layout for beneficiary company name
</commit_message>
<xml_diff>
--- a/backend/templates/payroll_template.xlsx
+++ b/backend/templates/payroll_template.xlsx
@@ -2,10 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29429"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC951805-3DE8-48C7-8C5B-2085647A2026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr filterPrivacy="true"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="Payroll Report" sheetId="1" r:id="rId1"/>
@@ -31,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>CÔNG TY CỔ PHẦN QUỐC TẾ THƯƠNG MẠI VÀ DỊCH VỤ VIỆT PHÁP</t>
   </si>
@@ -97,66 +96,75 @@
   </si>
   <si>
     <t>Số tiền</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0\ &quot;₫&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF323232"/>
       <sz val="11"/>
-      <color rgb="FF323232"/>
-      <name val="Arial"/>
     </font>
     <font>
-      <b/>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
     </font>
     <font>
-      <b/>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <name val="Arial"/>
       <sz val="11"/>
-      <name val="Arial"/>
     </font>
     <font>
-      <b/>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFF0000"/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF323232"/>
       <name val="Arial"/>
       <charset val="1"/>
+      <b val="1"/>
+      <color rgb="FF323232"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="7">
@@ -179,13 +187,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="0" tint="-0.1499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
+        <fgColor theme="5" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -238,103 +246,106 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" indent="1" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" indent="1" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="left" indent="1" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="right" indent="1" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="right" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="6"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="6"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment indent="2" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="left" indent="6" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment horizontal="left" indent="6" wrapText="true"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="true" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center" wrapText="true"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -347,51 +358,38 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
+<xdr:wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>257175</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>219075</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="3048000" cy="1219200"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D73BDFEA-77F9-846B-04BC-DD2B076F2AE1}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
+        <xdr:cNvPr id="3" name="TingTing Soft Banner" descr="TingTing Soft technology solutions banner"/>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks noChangeAspect="true"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="257175" y="2133600"/>
-          <a:ext cx="476250" cy="476250"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="3048000" cy="1219200"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
+        <a:prstGeom prst="rect"/>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:oneCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -443,7 +441,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -701,22 +699,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="26.28515625" style="7" customWidth="1"/>
-    <col min="4" max="4" width="22" style="1" customWidth="1"/>
-    <col min="5" max="5" width="38" style="7" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="5.85546875" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col customWidth="true" max="1" min="1" style="1" width="7.7109375"/>
+    <col customWidth="true" max="2" min="2" style="1" width="13.42578125"/>
+    <col customWidth="true" max="3" min="3" style="7" width="26.28515625"/>
+    <col customWidth="true" max="4" min="4" style="1" width="22"/>
+    <col customWidth="true" max="5" min="5" style="7" width="21.140625"/>
+    <col customWidth="true" max="6" min="6" style="1" width="15.140625"/>
+    <col customWidth="true" max="7" min="7" style="1" width="5.85546875"/>
+    <col max="16384" min="8" style="1" width="9.140625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="22.5" customHeight="1">
+    <row r="1" spans="1:6" ht="22.5" customHeight="true">
       <c r="B1" s="18" t="s">
         <v>0</v>
       </c>
@@ -727,7 +725,7 @@
       <c r="E1" s="23"/>
       <c r="F1" s="23"/>
     </row>
-    <row r="2" spans="1:6" ht="22.5" customHeight="1">
+    <row r="2" spans="1:6" ht="22.5" customHeight="true">
       <c r="A2" s="17"/>
       <c r="B2" s="18"/>
       <c r="C2" s="18"/>
@@ -737,7 +735,7 @@
       <c r="E2" s="28"/>
       <c r="F2" s="28"/>
     </row>
-    <row r="3" spans="1:6" ht="22.5" customHeight="1">
+    <row r="3" spans="1:6" ht="22.5" customHeight="true">
       <c r="A3" s="17"/>
       <c r="B3" s="18"/>
       <c r="C3" s="18"/>
@@ -747,7 +745,7 @@
       <c r="E3" s="29"/>
       <c r="F3" s="29"/>
     </row>
-    <row r="4" spans="1:6" ht="22.5" customHeight="1">
+    <row r="4" spans="1:6" ht="22.5" customHeight="true">
       <c r="A4" s="17"/>
       <c r="B4" s="17"/>
       <c r="C4" s="17"/>
@@ -760,7 +758,7 @@
       </c>
       <c r="F4" s="29"/>
     </row>
-    <row r="5" spans="1:6" ht="22.5" customHeight="1">
+    <row r="5" spans="1:6" ht="22.5" customHeight="true">
       <c r="A5" s="27"/>
       <c r="B5" s="27"/>
       <c r="C5" s="27"/>
@@ -773,7 +771,7 @@
       </c>
       <c r="F5" s="31"/>
     </row>
-    <row r="6" spans="1:6" ht="22.5" customHeight="1">
+    <row r="6" spans="1:6" ht="22.5" customHeight="true">
       <c r="A6" s="14"/>
       <c r="B6" s="14"/>
       <c r="C6" s="15"/>
@@ -783,7 +781,7 @@
       <c r="E6" s="21"/>
       <c r="F6" s="22"/>
     </row>
-    <row r="7" spans="1:6" ht="22.5" customHeight="1">
+    <row r="7" spans="1:6" ht="22.5" customHeight="true">
       <c r="A7" s="14"/>
       <c r="B7" s="14"/>
       <c r="C7" s="15"/>
@@ -791,10 +789,10 @@
       <c r="E7" s="10"/>
       <c r="F7" s="5"/>
     </row>
-    <row r="8" spans="1:6" ht="22.5" customHeight="1">
+    <row r="8" spans="1:6" ht="22.5" customHeight="true">
       <c r="A8" s="14"/>
       <c r="B8" s="20" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="C8" s="20"/>
       <c r="D8" s="23" t="s">
@@ -803,19 +801,19 @@
       <c r="E8" s="23"/>
       <c r="F8" s="23"/>
     </row>
-    <row r="9" spans="1:6" ht="22.5" customHeight="1">
+    <row r="9" spans="1:6" ht="32" customHeight="true">
       <c r="A9" s="16"/>
       <c r="B9" s="20"/>
       <c r="C9" s="20"/>
       <c r="D9" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="24" t="s">
+      <c r="E9" s="32" t="s">
         <v>10</v>
       </c>
       <c r="F9" s="24"/>
     </row>
-    <row r="10" spans="1:6" ht="22.5" customHeight="1">
+    <row r="10" spans="1:6" ht="22.5" customHeight="true">
       <c r="A10" s="16"/>
       <c r="B10" s="16"/>
       <c r="C10" s="16"/>
@@ -827,7 +825,7 @@
       </c>
       <c r="F10" s="21"/>
     </row>
-    <row r="11" spans="1:6" ht="22.5" customHeight="1">
+    <row r="11" spans="1:6" ht="22.5" customHeight="true">
       <c r="A11" s="16"/>
       <c r="B11" s="16"/>
       <c r="C11" s="16"/>
@@ -839,12 +837,12 @@
       </c>
       <c r="F11" s="26"/>
     </row>
-    <row r="12" spans="1:6" ht="22.5" customHeight="1">
+    <row r="12" spans="1:6" ht="22.5" customHeight="true">
       <c r="A12" s="14"/>
       <c r="B12" s="14"/>
       <c r="C12" s="15"/>
     </row>
-    <row r="13" spans="1:6" ht="22.5" customHeight="1">
+    <row r="13" spans="1:6" ht="22.5" customHeight="true">
       <c r="A13" s="19" t="s">
         <v>15</v>
       </c>
@@ -900,7 +898,7 @@
     <mergeCell ref="E5:F5"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait"/>
+  <pageSetup fitToHeight="0" orientation="portrait" paperSize="9"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(settings): configurable transfer bank info for statements
Admin-configurable beneficiary bank (holder, account number, bank name)
rendered into payroll statement emails and Excel attachments.

- New settings keys transfer_bank_account_{holder,number,name} with MB
  defaults (271866699, Ngân hàng Quân đội (MB))
- Email template placeholders {{.BankHolder}}/{{.BankNumber}}/{{.BankName}}
- Runtime cell overrides in all three Excel exporters; templates patched
  to MB defaults
- Settings page section with upsert save (creates rows on first save);
  account-number input mode with tabular digits
- PayrollReportPort.GenerateExcel gains ctx
</commit_message>
<xml_diff>
--- a/backend/templates/payroll_template.xlsx
+++ b/backend/templates/payroll_template.xlsx
@@ -68,13 +68,13 @@
     <t>Số Tài Khoản</t>
   </si>
   <si>
-    <t>283866888</t>
+    <t>271866699</t>
   </si>
   <si>
     <t>Ngân Hàng</t>
   </si>
   <si>
-    <t>TECHCOMBANK</t>
+    <t>Ngân hàng Quân đội (MB)</t>
   </si>
   <si>
     <t>CHI TIẾT GIAO DỊCH</t>

</xml_diff>